<commit_message>
Tracker: give the cancelled-row rule an explicit dark fill
Google Sheets exports a fill-less conditional format as white in Excel.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01C31xGpXxLcjXH3oTDRifkH
</commit_message>
<xml_diff>
--- a/products/hidden-cost-tracker/Hidden-Cost-Tracker.xlsx
+++ b/products/hidden-cost-tracker/Hidden-Cost-Tracker.xlsx
@@ -1038,6 +1038,11 @@
         <color rgb="006E6C80"/>
         <sz val="10"/>
       </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00262A3D"/>
+        </patternFill>
+      </fill>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>

</xml_diff>

<commit_message>
Fix styling lost in desktop Excel for all three trackers
openpyxl omits applyFill/applyNumberFormat flags and writes font name/size in
conditional-format styles; desktop Excel then drops fills and number formats.
Shared post-save fix in products/build/excel_compat.py.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01C31xGpXxLcjXH3oTDRifkH
</commit_message>
<xml_diff>
--- a/products/hidden-cost-tracker/Hidden-Cost-Tracker.xlsx
+++ b/products/hidden-cost-tracker/Hidden-Cost-Tracker.xlsx
@@ -595,255 +595,252 @@
   </cellStyleXfs>
   <cellXfs count="88">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyFill="1" numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf applyFill="1" applyFont="1" numFmtId="0" fontId="12" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf applyBorder="1" applyFill="1" applyFont="1" numFmtId="0" fontId="4" fillId="4" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="169" fontId="13" fillId="4" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyBorder="1" numFmtId="0" fontId="0" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf applyFill="1" applyFont="1" numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1" numFmtId="169" fontId="13" fillId="4" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyBorder="1" numFmtId="0" fontId="0" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf applyBorder="1" applyFill="1" applyFont="1" numFmtId="0" fontId="4" fillId="4" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom" indent="1"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="4" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1" numFmtId="164" fontId="14" fillId="4" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="15" fillId="4" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyBorder="1" numFmtId="0" fontId="0" fillId="0" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1" numFmtId="164" fontId="15" fillId="4" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="165" fontId="15" fillId="4" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1" numFmtId="165" fontId="15" fillId="4" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="4" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1" numFmtId="164" fontId="16" fillId="4" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyBorder="1" applyFill="1" applyFont="1" numFmtId="0" fontId="9" fillId="4" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" indent="1"/>
     </xf>
-    <xf numFmtId="165" fontId="17" fillId="4" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1" numFmtId="165" fontId="17" fillId="4" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="4" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1" numFmtId="164" fontId="17" fillId="4" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="1" fontId="18" fillId="4" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1" numFmtId="1" fontId="18" fillId="4" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyFill="1" applyFont="1" numFmtId="0" fontId="19" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyFill="1" applyFont="1" numFmtId="0" fontId="25" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="3" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyBorder="1" applyFill="1" applyFont="1" numFmtId="0" fontId="20" fillId="3" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyBorder="1" applyFill="1" applyFont="1" numFmtId="0" fontId="5" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1" numFmtId="164" fontId="5" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="170" fontId="5" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1" numFmtId="170" fontId="5" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="5" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1" numFmtId="168" fontId="5" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyBorder="1" applyFill="1" applyFont="1" numFmtId="0" fontId="5" fillId="7" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="7" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1" numFmtId="164" fontId="5" fillId="7" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="170" fontId="5" fillId="7" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1" numFmtId="170" fontId="5" fillId="7" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="5" fillId="7" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1" numFmtId="168" fontId="5" fillId="7" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyFill="1" applyFont="1" numFmtId="0" fontId="21" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="3" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyBorder="1" applyFill="1" applyFont="1" numFmtId="0" fontId="22" fillId="3" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyFill="1" applyFont="1" numFmtId="0" fontId="33" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyFill="1" applyFont="1" numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="5" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyBorder="1" applyFill="1" applyFont="1" numFmtId="0" fontId="34" fillId="5" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyFill="1" applyFont="1" numFmtId="0" fontId="23" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyBorder="1" applyFill="1" applyFont="1" numFmtId="0" fontId="24" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1" numFmtId="165" fontId="5" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyBorder="1" applyFill="1" applyFont="1" numFmtId="0" fontId="5" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="7" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1" numFmtId="165" fontId="5" fillId="7" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyBorder="1" applyFill="1" applyFont="1" numFmtId="0" fontId="5" fillId="7" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyBorder="1" applyFill="1" applyFont="1" numFmtId="0" fontId="10" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyBorder="1" applyFill="1" applyFont="1" numFmtId="0" fontId="11" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1" numFmtId="164" fontId="11" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="5" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1" numFmtId="9" fontId="5" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="8" fillId="7" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1" numFmtId="9" fontId="8" fillId="7" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="8" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1" numFmtId="9" fontId="8" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyBorder="1" applyFill="1" applyFont="1" numFmtId="0" fontId="26" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="26" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1" numFmtId="164" fontId="26" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="27" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1" numFmtId="9" fontId="27" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="7" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyBorder="1" applyFill="1" applyFont="1" numFmtId="0" fontId="28" fillId="7" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="28" fillId="7" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1" numFmtId="164" fontId="28" fillId="7" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="29" fillId="7" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1" numFmtId="9" fontId="29" fillId="7" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyFill="1" applyFont="1" numFmtId="0" fontId="30" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyFill="1" applyFont="1" numFmtId="0" fontId="23" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyFill="1" applyFont="1" numFmtId="0" fontId="31" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyFill="1" applyFont="1" numFmtId="0" fontId="21" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyFill="1" applyFont="1" numFmtId="0" fontId="32" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyFill="1" applyFont="1" numFmtId="0" fontId="9" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf applyFill="1" applyFont="1" numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf applyFill="1" applyFont="1" numFmtId="0" fontId="11" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyFill="1" applyFont="1" numFmtId="0" fontId="8" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyBorder="1" applyFill="1" applyFont="1" numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyBorder="1" applyFill="1" applyFont="1" numFmtId="0" fontId="4" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyBorder="1" numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf applyBorder="1" numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1" numFmtId="164" fontId="6" fillId="5" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="6" fillId="5" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyFill="1" applyFont="1" numFmtId="0" fontId="7" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1" numFmtId="165" fontId="6" fillId="5" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="6" fillId="5" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1" numFmtId="1" fontId="6" fillId="5" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="8" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1" numFmtId="166" fontId="8" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyBorder="1" applyFill="1" applyFont="1" numFmtId="0" fontId="5" fillId="5" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyBorder="1" applyFill="1" applyFont="1" numFmtId="0" fontId="5" fillId="6" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyFill="1" applyFont="1" numFmtId="0" fontId="11" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf applyBorder="1" applyFill="1" applyFont="1" numFmtId="0" fontId="5" fillId="5" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="5" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1" numFmtId="164" fontId="5" fillId="5" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="5" fillId="5" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1" numFmtId="1" fontId="5" fillId="5" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="5" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1" numFmtId="165" fontId="5" fillId="5" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="5" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1" numFmtId="1" fontId="5" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1" numFmtId="166" fontId="5" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyBorder="1" applyFill="1" applyFont="1" numFmtId="0" fontId="5" fillId="6" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="6" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1" numFmtId="164" fontId="5" fillId="6" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="5" fillId="6" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1" numFmtId="1" fontId="5" fillId="6" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="6" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1" numFmtId="165" fontId="5" fillId="6" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="5" fillId="7" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1" numFmtId="1" fontId="5" fillId="7" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="7" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1" numFmtId="166" fontId="5" fillId="7" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="5" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1" numFmtId="166" fontId="5" fillId="5" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="6" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1" numFmtId="166" fontId="5" fillId="6" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyBorder="1" applyFill="1" applyFont="1" numFmtId="0" fontId="5" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="16">
+  <dxfs count="13">
     <dxf>
       <font>
-        <name val="Arial"/>
         <b val="1"/>
-        <strike val="0"/>
         <color rgb="00F2B544"/>
-        <sz val="10"/>
       </font>
       <fill>
         <patternFill patternType="solid">
@@ -853,11 +850,8 @@
     </dxf>
     <dxf>
       <font>
-        <name val="Arial"/>
         <b val="1"/>
-        <strike val="0"/>
         <color rgb="00FF6B6B"/>
-        <sz val="10"/>
       </font>
       <fill>
         <patternFill patternType="solid">
@@ -867,39 +861,8 @@
     </dxf>
     <dxf>
       <font>
-        <name val="Arial"/>
         <b val="1"/>
-        <strike val="0"/>
-        <color rgb="00FF6B6B"/>
-        <sz val="9"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="004A1D22"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <b val="1"/>
-        <strike val="0"/>
-        <color rgb="00F2B544"/>
-        <sz val="9"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="004A3A15"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <b val="1"/>
-        <strike val="0"/>
         <color rgb="005FD38D"/>
-        <sz val="9"/>
       </font>
       <fill>
         <patternFill patternType="solid">
@@ -909,11 +872,8 @@
     </dxf>
     <dxf>
       <font>
-        <name val="Arial"/>
         <b val="1"/>
-        <strike val="0"/>
         <color rgb="008AB4FF"/>
-        <sz val="9"/>
       </font>
       <fill>
         <patternFill patternType="solid">
@@ -923,11 +883,8 @@
     </dxf>
     <dxf>
       <font>
-        <name val="Arial"/>
         <b val="1"/>
-        <strike val="0"/>
         <color rgb="00F06BC8"/>
-        <sz val="9"/>
       </font>
       <fill>
         <patternFill patternType="solid">
@@ -937,11 +894,8 @@
     </dxf>
     <dxf>
       <font>
-        <name val="Arial"/>
         <b val="1"/>
-        <strike val="0"/>
         <color rgb="004FC3C7"/>
-        <sz val="9"/>
       </font>
       <fill>
         <patternFill patternType="solid">
@@ -951,11 +905,8 @@
     </dxf>
     <dxf>
       <font>
-        <name val="Arial"/>
         <b val="1"/>
-        <strike val="0"/>
         <color rgb="00B8B6C8"/>
-        <sz val="9"/>
       </font>
       <fill>
         <patternFill patternType="solid">
@@ -965,20 +916,14 @@
     </dxf>
     <dxf>
       <font>
-        <name val="Arial"/>
         <b val="1"/>
-        <strike val="0"/>
         <color rgb="00FF6B6B"/>
-        <sz val="10"/>
       </font>
     </dxf>
     <dxf>
       <font>
-        <name val="Arial"/>
         <b val="1"/>
-        <strike val="0"/>
         <color rgb="00F08A4B"/>
-        <sz val="10"/>
       </font>
       <fill>
         <patternFill patternType="solid">
@@ -988,25 +933,8 @@
     </dxf>
     <dxf>
       <font>
-        <name val="Arial"/>
         <b val="1"/>
-        <strike val="0"/>
-        <color rgb="00F08A4B"/>
-        <sz val="9"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="004A2A18"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <b val="1"/>
-        <strike val="0"/>
         <color rgb="00B18CFF"/>
-        <sz val="9"/>
       </font>
       <fill>
         <patternFill patternType="solid">
@@ -1016,11 +944,8 @@
     </dxf>
     <dxf>
       <font>
-        <name val="Arial"/>
         <b val="1"/>
-        <strike val="0"/>
         <color rgb="00F2B544"/>
-        <sz val="10"/>
       </font>
     </dxf>
     <dxf>
@@ -1032,11 +957,7 @@
     </dxf>
     <dxf>
       <font>
-        <name val="Arial"/>
-        <i val="1"/>
-        <strike val="1"/>
         <color rgb="006E6C80"/>
-        <sz val="10"/>
       </font>
       <fill>
         <patternFill patternType="solid">
@@ -3391,13 +3312,13 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D31:D36">
-    <cfRule type="cellIs" priority="4" operator="equal" dxfId="2">
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="1">
       <formula>"HIGH"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="5" operator="equal" dxfId="3">
+    <cfRule type="cellIs" priority="5" operator="equal" dxfId="0">
       <formula>"CHECK"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="6" operator="equal" dxfId="4">
+    <cfRule type="cellIs" priority="6" operator="equal" dxfId="2">
       <formula>"OK"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5481,43 +5402,43 @@
   </sheetData>
   <autoFilter ref="B5:R25"/>
   <conditionalFormatting sqref="C6:C25">
-    <cfRule type="cellIs" priority="1" operator="equal" dxfId="2">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="1">
       <formula>"Credit card"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="2" operator="equal" dxfId="5">
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="3">
       <formula>"Loan"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" dxfId="3">
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="0">
       <formula>"Installment"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" dxfId="6">
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="4">
       <formula>"BNPL"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="5" operator="equal" dxfId="7">
+    <cfRule type="cellIs" priority="5" operator="equal" dxfId="5">
       <formula>"Family / friend"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="6" operator="equal" dxfId="8">
+    <cfRule type="cellIs" priority="6" operator="equal" dxfId="6">
       <formula>"Other"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="R6:R25">
-    <cfRule type="cellIs" priority="7" operator="equal" dxfId="2">
+    <cfRule type="cellIs" priority="7" operator="equal" dxfId="1">
       <formula>"HIGH"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="8" operator="equal" dxfId="3">
+    <cfRule type="cellIs" priority="8" operator="equal" dxfId="0">
       <formula>"CHECK"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="9" operator="equal" dxfId="4">
+    <cfRule type="cellIs" priority="9" operator="equal" dxfId="2">
       <formula>"OK"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J6:J25">
-    <cfRule type="expression" priority="10" dxfId="9">
+    <cfRule type="expression" priority="10" dxfId="7">
       <formula>AND(ISNUMBER($J6),$J6&gt;=Settings!$C$6)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P6:P25">
-    <cfRule type="cellIs" priority="11" operator="equal" dxfId="10">
+    <cfRule type="cellIs" priority="11" operator="equal" dxfId="8">
       <formula>1</formula>
     </cfRule>
   </conditionalFormatting>
@@ -8062,86 +7983,86 @@
   </sheetData>
   <autoFilter ref="B5:R35"/>
   <conditionalFormatting sqref="C6:C35">
-    <cfRule type="cellIs" priority="1" operator="equal" dxfId="6">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="4">
       <formula>"Streaming"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="2" operator="equal" dxfId="5">
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="3">
       <formula>"Software"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" dxfId="4">
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="2">
       <formula>"Fitness"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" dxfId="11">
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="8">
       <formula>"Shopping"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="5" operator="equal" dxfId="8">
+    <cfRule type="cellIs" priority="5" operator="equal" dxfId="6">
       <formula>"News"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="6" operator="equal" dxfId="7">
+    <cfRule type="cellIs" priority="6" operator="equal" dxfId="5">
       <formula>"Cloud"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="7" operator="equal" dxfId="3">
+    <cfRule type="cellIs" priority="7" operator="equal" dxfId="0">
       <formula>"Food"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="8" operator="equal" dxfId="12">
+    <cfRule type="cellIs" priority="8" operator="equal" dxfId="9">
       <formula>"Education"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="9" operator="equal" dxfId="8">
+    <cfRule type="cellIs" priority="9" operator="equal" dxfId="6">
       <formula>"Other"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E6:E35">
-    <cfRule type="cellIs" priority="10" operator="equal" dxfId="6">
+    <cfRule type="cellIs" priority="10" operator="equal" dxfId="4">
       <formula>"Weekly"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="11" operator="equal" dxfId="12">
+    <cfRule type="cellIs" priority="11" operator="equal" dxfId="9">
       <formula>"Monthly"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="12" operator="equal" dxfId="7">
+    <cfRule type="cellIs" priority="12" operator="equal" dxfId="5">
       <formula>"Quarterly"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="13" operator="equal" dxfId="3">
+    <cfRule type="cellIs" priority="13" operator="equal" dxfId="0">
       <formula>"Yearly"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H6:H35">
-    <cfRule type="cellIs" priority="14" operator="equal" dxfId="4">
+    <cfRule type="cellIs" priority="14" operator="equal" dxfId="2">
       <formula>"Yes"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="15" operator="equal" dxfId="8">
+    <cfRule type="cellIs" priority="15" operator="equal" dxfId="6">
       <formula>"No"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I6:I35">
-    <cfRule type="cellIs" priority="16" operator="equal" dxfId="2">
+    <cfRule type="cellIs" priority="16" operator="equal" dxfId="1">
       <formula>"Yes"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="17" operator="equal" dxfId="8">
+    <cfRule type="cellIs" priority="17" operator="equal" dxfId="6">
       <formula>"No"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J6:J35">
-    <cfRule type="cellIs" priority="18" operator="equal" dxfId="3">
+    <cfRule type="cellIs" priority="18" operator="equal" dxfId="0">
       <formula>"Yes"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="19" operator="equal" dxfId="8">
+    <cfRule type="cellIs" priority="19" operator="equal" dxfId="6">
       <formula>"No"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="R6:R35">
-    <cfRule type="cellIs" priority="20" operator="equal" dxfId="2">
+    <cfRule type="cellIs" priority="20" operator="equal" dxfId="1">
       <formula>"Cancel soon?"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="21" operator="equal" dxfId="2">
+    <cfRule type="cellIs" priority="21" operator="equal" dxfId="1">
       <formula>"Trial ended"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="22" operator="equal" dxfId="3">
+    <cfRule type="cellIs" priority="22" operator="equal" dxfId="0">
       <formula>"Charge soon"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="23" operator="equal" dxfId="8">
+    <cfRule type="cellIs" priority="23" operator="equal" dxfId="6">
       <formula>"To cancel"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="24" operator="equal" dxfId="4">
+    <cfRule type="cellIs" priority="24" operator="equal" dxfId="2">
       <formula>"OK"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -8151,17 +8072,17 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O6:O35">
-    <cfRule type="expression" priority="26" dxfId="13">
+    <cfRule type="expression" priority="26" dxfId="10">
       <formula>AND(ISNUMBER($O6),$O6&lt;=Settings!$C$8)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B6:G35">
-    <cfRule type="expression" priority="27" dxfId="14">
+    <cfRule type="expression" priority="27" dxfId="11">
       <formula>$R6="Cancel soon?"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B6:Q35">
-    <cfRule type="expression" priority="28" dxfId="15">
+    <cfRule type="expression" priority="28" dxfId="12">
       <formula>$I6="Yes"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>